<commit_message>
committing code to update github index
</commit_message>
<xml_diff>
--- a/processed-data/09_xenium_panel/Amygdala_Xenium_panel.xlsx
+++ b/processed-data/09_xenium_panel/Amygdala_Xenium_panel.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="200" uniqueCount="132">
   <si>
     <t>Region</t>
   </si>
@@ -110,6 +110,303 @@
   </si>
   <si>
     <t>FOXP2</t>
+  </si>
+  <si>
+    <t>Excit_1</t>
+  </si>
+  <si>
+    <t>TMEM132C</t>
+  </si>
+  <si>
+    <t>BTBD11</t>
+  </si>
+  <si>
+    <t>HGF</t>
+  </si>
+  <si>
+    <t>MCOLN3</t>
+  </si>
+  <si>
+    <t>PWRN4</t>
+  </si>
+  <si>
+    <t>Excit_2</t>
+  </si>
+  <si>
+    <t>TESPA1</t>
+  </si>
+  <si>
+    <t>SEMA6D</t>
+  </si>
+  <si>
+    <t>NTNG1</t>
+  </si>
+  <si>
+    <t>CUX2</t>
+  </si>
+  <si>
+    <t>Excit_3</t>
+  </si>
+  <si>
+    <t>TOX3</t>
+  </si>
+  <si>
+    <t>LAMA3</t>
+  </si>
+  <si>
+    <t>Excit_4</t>
+  </si>
+  <si>
+    <t>SLC38A11</t>
+  </si>
+  <si>
+    <t>DCSTAMP</t>
+  </si>
+  <si>
+    <t>COBLL1</t>
+  </si>
+  <si>
+    <t>Excit_5</t>
+  </si>
+  <si>
+    <t>NPFFR2</t>
+  </si>
+  <si>
+    <t>PRSS12</t>
+  </si>
+  <si>
+    <t>Excit_6</t>
+  </si>
+  <si>
+    <t>VAV3</t>
+  </si>
+  <si>
+    <t>RXFP2</t>
+  </si>
+  <si>
+    <t>POU6F2</t>
+  </si>
+  <si>
+    <t>ECE2</t>
+  </si>
+  <si>
+    <t>Excit_7</t>
+  </si>
+  <si>
+    <t>SATB2</t>
+  </si>
+  <si>
+    <t>MPPED1</t>
+  </si>
+  <si>
+    <t>FAM163A</t>
+  </si>
+  <si>
+    <t>BTC</t>
+  </si>
+  <si>
+    <t>TWIST1</t>
+  </si>
+  <si>
+    <t>Excit_8</t>
+  </si>
+  <si>
+    <t>UST</t>
+  </si>
+  <si>
+    <t>SEMA3E</t>
+  </si>
+  <si>
+    <t>CDH6</t>
+  </si>
+  <si>
+    <t>VWA2</t>
+  </si>
+  <si>
+    <t>CLMP</t>
+  </si>
+  <si>
+    <t>HCRTR2</t>
+  </si>
+  <si>
+    <t>SHB</t>
+  </si>
+  <si>
+    <t>Excit_9</t>
+  </si>
+  <si>
+    <t>CALCRL</t>
+  </si>
+  <si>
+    <t>BCHE</t>
+  </si>
+  <si>
+    <t>Excit_10</t>
+  </si>
+  <si>
+    <t>THEMIS</t>
+  </si>
+  <si>
+    <t>Excit_11</t>
+  </si>
+  <si>
+    <t>CTXND1</t>
+  </si>
+  <si>
+    <t>MET</t>
+  </si>
+  <si>
+    <t>POU3F1</t>
+  </si>
+  <si>
+    <t>ST8SIA2</t>
+  </si>
+  <si>
+    <t>FEZF2</t>
+  </si>
+  <si>
+    <t>Excit_12</t>
+  </si>
+  <si>
+    <t>ADRA1A</t>
+  </si>
+  <si>
+    <t>PRLR</t>
+  </si>
+  <si>
+    <t>ITC_1</t>
+  </si>
+  <si>
+    <t>MEIS2</t>
+  </si>
+  <si>
+    <t>KIRREL1</t>
+  </si>
+  <si>
+    <t>SV2C</t>
+  </si>
+  <si>
+    <t>GRIK3</t>
+  </si>
+  <si>
+    <t>CDH12</t>
+  </si>
+  <si>
+    <t>ITC_2</t>
+  </si>
+  <si>
+    <t>ADAMTSL1</t>
+  </si>
+  <si>
+    <t>PREX2</t>
+  </si>
+  <si>
+    <t>LAMP5_1</t>
+  </si>
+  <si>
+    <t>PRR16</t>
+  </si>
+  <si>
+    <t>FRAS1</t>
+  </si>
+  <si>
+    <t>LAMP5_2</t>
+  </si>
+  <si>
+    <t>CHST9</t>
+  </si>
+  <si>
+    <t>SORCS1</t>
+  </si>
+  <si>
+    <t>PVALB</t>
+  </si>
+  <si>
+    <t>LHX6</t>
+  </si>
+  <si>
+    <t>VIP_1</t>
+  </si>
+  <si>
+    <t>RYR3</t>
+  </si>
+  <si>
+    <t>GRIK1</t>
+  </si>
+  <si>
+    <t>VIP_2</t>
+  </si>
+  <si>
+    <t>SOX5</t>
+  </si>
+  <si>
+    <t>ZBTB20</t>
+  </si>
+  <si>
+    <t>Inh_4</t>
+  </si>
+  <si>
+    <t>ST18</t>
+  </si>
+  <si>
+    <t>Inh_5</t>
+  </si>
+  <si>
+    <t>ADAMTS5</t>
+  </si>
+  <si>
+    <t>Inh_3</t>
+  </si>
+  <si>
+    <t>PCDH18</t>
+  </si>
+  <si>
+    <t>Inh_2</t>
+  </si>
+  <si>
+    <t>DOCK8</t>
+  </si>
+  <si>
+    <t>Inh_1</t>
+  </si>
+  <si>
+    <t>ANO2</t>
+  </si>
+  <si>
+    <t>CEA</t>
+  </si>
+  <si>
+    <t>GPR149</t>
+  </si>
+  <si>
+    <t>RARB</t>
+  </si>
+  <si>
+    <t>CCDC88C</t>
+  </si>
+  <si>
+    <t>LPL</t>
+  </si>
+  <si>
+    <t>ONECUT2</t>
+  </si>
+  <si>
+    <t>MEA</t>
+  </si>
+  <si>
+    <t>TMEM108</t>
+  </si>
+  <si>
+    <t>NHS</t>
+  </si>
+  <si>
+    <t>DNER</t>
+  </si>
+  <si>
+    <t>PLCB4</t>
+  </si>
+  <si>
+    <t>KCNJ3</t>
   </si>
 </sst>
 </file>
@@ -154,7 +451,18 @@
   <cellStyles count="1">
     <cellStyle xfId="0" name="Normal" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="1">
+    <dxf>
+      <font/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFB7E1CD"/>
+          <bgColor rgb="FFB7E1CD"/>
+        </patternFill>
+      </fill>
+      <border/>
+    </dxf>
+  </dxfs>
 </styleSheet>
 </file>
 
@@ -533,10 +841,10 @@
     </row>
     <row r="22">
       <c r="A22" s="1" t="s">
-        <v>21</v>
+        <v>26</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
     </row>
     <row r="23">
@@ -544,7 +852,7 @@
         <v>26</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="24">
@@ -552,7 +860,7 @@
         <v>26</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
     </row>
     <row r="25">
@@ -560,7 +868,7 @@
         <v>26</v>
       </c>
       <c r="B25" s="1" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
     <row r="26">
@@ -568,7 +876,7 @@
         <v>26</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
     <row r="27">
@@ -576,18 +884,599 @@
         <v>26</v>
       </c>
       <c r="B27" s="1" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="1" t="s">
-        <v>26</v>
+        <v>33</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>32</v>
+        <v>34</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="B29" s="1" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="B30" s="1" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="B31" s="1" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="B32" s="1" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="B33" s="1" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="B34" s="1" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="B35" s="1" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="B36" s="1" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="B37" s="1" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="B38" s="1" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="B39" s="1" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="B40" s="1" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="B41" s="1" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="B42" s="1" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="B43" s="1" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="B44" s="1" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="B45" s="1" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="B46" s="1" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="B47" s="1" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="B48" s="1" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="B49" s="1" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="B50" s="1" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="B51" s="1" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="B52" s="1" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="B53" s="1" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="B54" s="1" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="B55" s="1" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="B56" s="1" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="B57" s="1" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="B58" s="1" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="B59" s="1" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="B60" s="1" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="B61" s="1" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="B62" s="1" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="B63" s="1" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="B64" s="1" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="B65" s="1" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="B66" s="1" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="B67" s="1" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="B68" s="1" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="B69" s="1" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="B70" s="1" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="B71" s="1" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="B72" s="1" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="B73" s="1" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="B74" s="1" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="B75" s="1" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="B76" s="1" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="B77" s="1" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="B78" s="1" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="B79" s="1" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="B80" s="1" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="1" t="s">
+        <v>102</v>
+      </c>
+      <c r="B81" s="1" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="B82" s="1" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="B83" s="1" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="1" t="s">
+        <v>107</v>
+      </c>
+      <c r="B84" s="1" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="1" t="s">
+        <v>107</v>
+      </c>
+      <c r="B85" s="1" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="1" t="s">
+        <v>110</v>
+      </c>
+      <c r="B86" s="1" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="1" t="s">
+        <v>112</v>
+      </c>
+      <c r="B87" s="1" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="B88" s="1" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="B89" s="1" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="1" t="s">
+        <v>118</v>
+      </c>
+      <c r="B90" s="1" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="1" t="s">
+        <v>120</v>
+      </c>
+      <c r="B91" s="1" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="1" t="s">
+        <v>120</v>
+      </c>
+      <c r="B92" s="1" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="1" t="s">
+        <v>120</v>
+      </c>
+      <c r="B93" s="1" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="1" t="s">
+        <v>120</v>
+      </c>
+      <c r="B94" s="1" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="1" t="s">
+        <v>120</v>
+      </c>
+      <c r="B95" s="1" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="1" t="s">
+        <v>126</v>
+      </c>
+      <c r="B96" s="1" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="1" t="s">
+        <v>126</v>
+      </c>
+      <c r="B97" s="1" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="1" t="s">
+        <v>126</v>
+      </c>
+      <c r="B98" s="1" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="1" t="s">
+        <v>126</v>
+      </c>
+      <c r="B99" s="1" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" s="1" t="s">
+        <v>126</v>
+      </c>
+      <c r="B100" s="1" t="s">
+        <v>131</v>
       </c>
     </row>
   </sheetData>
+  <conditionalFormatting sqref="B1:B998">
+    <cfRule type="expression" dxfId="0" priority="1">
+      <formula>COUNTIF (B:B, B1)&gt;1</formula>
+    </cfRule>
+  </conditionalFormatting>
   <drawing r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>